<commit_message>
🔄 更新看板 08/10 11:06
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -1498,9 +1498,19 @@
           <t>13.6%</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>1412376</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>-41.0%</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>-36.1%</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
     </row>
@@ -1534,9 +1544,19 @@
           <t>21.1%</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>958914</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>+81.4%</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>+137.9%</t>
+        </is>
+      </c>
       <c r="M22" t="n">
         <v>43424</v>
       </c>
@@ -1578,9 +1598,19 @@
           <t>17.9%</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>2892074</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>-11.0%</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>+2.9%</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🔄 更新看板 08/10 11:09
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -1545,16 +1545,16 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>958914</v>
+        <v>1479698</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>+81.4%</t>
+          <t>+17.5%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>+137.9%</t>
+          <t>+31.5%</t>
         </is>
       </c>
       <c r="M22" t="n">

</xml_diff>

<commit_message>
🔄 更新看板 08/10 13:20
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -668,11 +668,11 @@
         <v>-46215</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>39588</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1486,11 +1486,11 @@
         <v>544651</v>
       </c>
       <c r="G21" t="n">
-        <v>37194</v>
+        <v>76782</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>14.2%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1586,11 +1586,11 @@
         <v>2076133</v>
       </c>
       <c r="G23" t="n">
-        <v>37194</v>
+        <v>76782</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1614,7 +1614,7 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>含协同37194元 | 普陀明细456896元 | 康博嘉43424元 | 退费率19.3%</t>
+          <t>含协同76782元 | 普陀明细456896元 | 康博嘉43424元 | 退费率19.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 更新看板 08/11 10:07
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -503,38 +503,38 @@
         <v>1000000</v>
       </c>
       <c r="D2" t="n">
-        <v>74781</v>
+        <v>77011</v>
       </c>
       <c r="E2" t="n">
-        <v>43382</v>
+        <v>44005</v>
       </c>
       <c r="F2" t="n">
-        <v>31399</v>
+        <v>33005</v>
       </c>
       <c r="G2" t="n">
         <v>8000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>306228</v>
+        <v>308000</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>-75.6%</t>
+          <t>-75.0%</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>-75.5%</t>
+          <t>-74.0%</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -555,38 +555,38 @@
         <v>100000</v>
       </c>
       <c r="D3" t="n">
-        <v>14430</v>
+        <v>18785</v>
       </c>
       <c r="E3" t="n">
-        <v>18154</v>
+        <v>24874</v>
       </c>
       <c r="F3" t="n">
-        <v>-3724</v>
+        <v>-6089</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>39885</v>
+        <v>41395</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>-63.8%</t>
+          <t>-54.6%</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>-120.0%</t>
+          <t>-142.9%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -607,38 +607,38 @@
         <v>800000</v>
       </c>
       <c r="D4" t="n">
-        <v>163371</v>
+        <v>197067</v>
       </c>
       <c r="E4" t="n">
-        <v>30315</v>
+        <v>81119</v>
       </c>
       <c r="F4" t="n">
-        <v>133055</v>
+        <v>115947</v>
       </c>
       <c r="G4" t="n">
         <v>10398</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>24.6%</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>207350</v>
+        <v>225139</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>-21.2%</t>
+          <t>-12.5%</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>-15.0%</t>
+          <t>-33.4%</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -659,29 +659,29 @@
         <v>650000</v>
       </c>
       <c r="D5" t="n">
-        <v>22943</v>
+        <v>23309</v>
       </c>
       <c r="E5" t="n">
         <v>69159</v>
       </c>
       <c r="F5" t="n">
-        <v>-46215</v>
+        <v>-45849</v>
       </c>
       <c r="G5" t="n">
         <v>39588</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>3.6%</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>278889</v>
+        <v>284571</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>-117.5%</t>
+          <t>-117.3%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -711,38 +711,38 @@
         <v>700000</v>
       </c>
       <c r="D6" t="n">
-        <v>117284</v>
+        <v>135037</v>
       </c>
       <c r="E6" t="n">
-        <v>15437</v>
+        <v>41016</v>
       </c>
       <c r="F6" t="n">
-        <v>101846</v>
+        <v>94020</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>26391</v>
+        <v>32521</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>+344.4%</t>
+          <t>+315.2%</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>+570.6%</t>
+          <t>+414.9%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -763,38 +763,38 @@
         <v>550000</v>
       </c>
       <c r="D7" t="n">
-        <v>91112</v>
+        <v>117462</v>
       </c>
       <c r="E7" t="n">
-        <v>37261</v>
+        <v>37267</v>
       </c>
       <c r="F7" t="n">
-        <v>53851</v>
+        <v>80195</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>182040</v>
+        <v>182211</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>-49.9%</t>
+          <t>-35.5%</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>-62.5%</t>
+          <t>-23.6%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -815,38 +815,38 @@
         <v>650000</v>
       </c>
       <c r="D8" t="n">
-        <v>78852</v>
+        <v>169398</v>
       </c>
       <c r="E8" t="n">
-        <v>14960</v>
+        <v>15007</v>
       </c>
       <c r="F8" t="n">
-        <v>63892</v>
+        <v>154391</v>
       </c>
       <c r="G8" t="n">
         <v>18796</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>29.0%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>100310</v>
+        <v>114620</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>-21.4%</t>
+          <t>+47.8%</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>+35.1%</t>
+          <t>+199.6%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -867,38 +867,38 @@
         <v>1700000</v>
       </c>
       <c r="D9" t="n">
-        <v>270721</v>
+        <v>317341</v>
       </c>
       <c r="E9" t="n">
-        <v>60174</v>
+        <v>53574</v>
       </c>
       <c r="F9" t="n">
-        <v>210547</v>
+        <v>263767</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>271283</v>
+        <v>295883</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>-0.2%</t>
+          <t>+7.3%</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>+168.9%</t>
+          <t>+195.5%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -919,23 +919,23 @@
         <v>2000000</v>
       </c>
       <c r="D10" t="n">
-        <v>502848</v>
+        <v>563265</v>
       </c>
       <c r="E10" t="n">
         <v>19</v>
       </c>
       <c r="F10" t="n">
-        <v>502829</v>
+        <v>563246</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -943,18 +943,18 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>+1108.9%</t>
+          <t>+1254.1%</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>+1237.4%</t>
+          <t>+1528.0%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>含普陀明细(456896元)</t>
+          <t>含普陀明细(517294元)</t>
         </is>
       </c>
     </row>
@@ -973,36 +973,36 @@
         <v>700000</v>
       </c>
       <c r="D11" t="n">
-        <v>199696</v>
+        <v>214684</v>
       </c>
       <c r="E11" t="n">
-        <v>1800</v>
+        <v>8800</v>
       </c>
       <c r="F11" t="n">
-        <v>197896</v>
+        <v>205884</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>30.7%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>30.7%</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>167496</v>
+        <v>187913</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>+19.2%</t>
+          <t>+14.2%</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>+43.9%</t>
+          <t>+31.9%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1023,36 +1023,36 @@
         <v>450000</v>
       </c>
       <c r="D12" t="n">
-        <v>35614</v>
+        <v>38614</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>35614</v>
+        <v>38605</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>126788</v>
+        <v>127784</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>-71.9%</t>
+          <t>-69.8%</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>-62.5%</t>
+          <t>-59.8%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1073,36 +1073,36 @@
         <v>800000</v>
       </c>
       <c r="D13" t="n">
-        <v>214431</v>
+        <v>223068</v>
       </c>
       <c r="E13" t="n">
-        <v>4056</v>
+        <v>14056</v>
       </c>
       <c r="F13" t="n">
-        <v>210375</v>
+        <v>209012</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>64911</v>
+        <v>127816</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>+230.3%</t>
+          <t>+74.5%</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>-7776.0%</t>
+          <t>-700.9%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1123,36 +1123,36 @@
         <v>850000</v>
       </c>
       <c r="D14" t="n">
-        <v>180041</v>
+        <v>190041</v>
       </c>
       <c r="E14" t="n">
         <v>25781</v>
       </c>
       <c r="F14" t="n">
-        <v>154260</v>
+        <v>164260</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>118398</v>
+        <v>139236</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>+52.1%</t>
+          <t>+36.5%</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>+75.9%</t>
+          <t>+72.0%</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1175,23 +1175,23 @@
         <v>450000</v>
       </c>
       <c r="D15" t="n">
-        <v>86520</v>
+        <v>126918</v>
       </c>
       <c r="E15" t="n">
         <v>299</v>
       </c>
       <c r="F15" t="n">
-        <v>86221</v>
+        <v>126619</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>+18.5%</t>
+          <t>+73.9%</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>+34.8%</t>
+          <t>+120.7%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1225,40 +1225,40 @@
         <v>700000</v>
       </c>
       <c r="D16" t="n">
-        <v>164643</v>
+        <v>166547</v>
       </c>
       <c r="E16" t="n">
         <v>299</v>
       </c>
       <c r="F16" t="n">
-        <v>164344</v>
+        <v>166248</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>129370</v>
+        <v>129968</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>+27.3%</t>
+          <t>+28.1%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>+41.0%</t>
+          <t>+41.9%</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>22900</v>
+        <v>23201</v>
       </c>
       <c r="N16" t="inlineStr"/>
     </row>
@@ -1277,40 +1277,40 @@
         <v>850000</v>
       </c>
       <c r="D17" t="n">
-        <v>117915</v>
+        <v>123246</v>
       </c>
       <c r="E17" t="n">
-        <v>143159</v>
+        <v>143178</v>
       </c>
       <c r="F17" t="n">
-        <v>-25243</v>
+        <v>-19931</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>115294</v>
+        <v>142512</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>+2.3%</t>
+          <t>-13.5%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>-131.9%</t>
+          <t>-118.7%</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>4143</v>
+        <v>4726</v>
       </c>
       <c r="N17" t="inlineStr"/>
     </row>
@@ -1329,23 +1329,23 @@
         <v>800000</v>
       </c>
       <c r="D18" t="n">
-        <v>96514</v>
+        <v>97456</v>
       </c>
       <c r="E18" t="n">
         <v>16937</v>
       </c>
       <c r="F18" t="n">
-        <v>79577</v>
+        <v>80519</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -1353,16 +1353,16 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>+26.6%</t>
+          <t>+27.9%</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>+592.6%</t>
+          <t>+895.2%</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>13098</v>
+        <v>13642</v>
       </c>
       <c r="N18" t="inlineStr"/>
     </row>
@@ -1381,23 +1381,23 @@
         <v>260000</v>
       </c>
       <c r="D19" t="n">
-        <v>98788</v>
+        <v>110788</v>
       </c>
       <c r="E19" t="n">
         <v>15277</v>
       </c>
       <c r="F19" t="n">
-        <v>83511</v>
+        <v>95511</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>42.6%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>42.6%</t>
         </is>
       </c>
       <c r="J19" t="n">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>+522.4%</t>
+          <t>+598.0%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>+428.0%</t>
+          <t>+503.9%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1431,36 +1431,36 @@
         <v>400000</v>
       </c>
       <c r="D20" t="n">
-        <v>42095</v>
+        <v>50693</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>42095</v>
+        <v>50693</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>29988</v>
+        <v>41988</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>+40.4%</t>
+          <t>+20.7%</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>+2374.7%</t>
+          <t>+270.0%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -1477,38 +1477,38 @@
         <v>6150000</v>
       </c>
       <c r="D21" t="n">
-        <v>833494</v>
+        <v>1055410</v>
       </c>
       <c r="E21" t="n">
-        <v>288842</v>
+        <v>366021</v>
       </c>
       <c r="F21" t="n">
-        <v>544651</v>
+        <v>689387</v>
       </c>
       <c r="G21" t="n">
         <v>76782</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1412376</v>
+        <v>1484340</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-41.0%</t>
+          <t>-28.9%</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-36.1%</t>
+          <t>-18.4%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -1525,44 +1525,44 @@
         <v>8260000</v>
       </c>
       <c r="D22" t="n">
-        <v>1739105</v>
+        <v>1905320</v>
       </c>
       <c r="E22" t="n">
-        <v>207627</v>
+        <v>224655</v>
       </c>
       <c r="F22" t="n">
-        <v>1531479</v>
+        <v>1680666</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1479698</v>
+        <v>1655887</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>+17.5%</t>
+          <t>+15.1%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>+31.5%</t>
+          <t>+38.0%</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>43424</v>
+        <v>44852</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>康博嘉5店(深圳13098,广州3283,武汉4143,杭州22900)</t>
+          <t>康博嘉5店(武汉4726,深圳13642,杭州23201,广州3283)</t>
         </is>
       </c>
     </row>
@@ -1577,44 +1577,44 @@
         <v>14410000</v>
       </c>
       <c r="D23" t="n">
-        <v>2572604</v>
+        <v>2960734</v>
       </c>
       <c r="E23" t="n">
-        <v>496470</v>
+        <v>590677</v>
       </c>
       <c r="F23" t="n">
-        <v>2076133</v>
+        <v>2370056</v>
       </c>
       <c r="G23" t="n">
         <v>76782</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2892074</v>
+        <v>3140227</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>-11.0%</t>
+          <t>-5.7%</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>+2.9%</t>
+          <t>+14.9%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>含协同76782元 | 普陀明细456896元 | 康博嘉43424元 | 退费率19.3%</t>
+          <t>含协同76782元 | 普陀明细517294元 | 康博嘉44852元 | 退费率20.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 更新看板 08/12 10:40
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -503,38 +503,38 @@
         <v>1000000</v>
       </c>
       <c r="D2" t="n">
-        <v>77011</v>
+        <v>79688</v>
       </c>
       <c r="E2" t="n">
-        <v>44005</v>
+        <v>73989</v>
       </c>
       <c r="F2" t="n">
-        <v>33005</v>
+        <v>5698</v>
       </c>
       <c r="G2" t="n">
         <v>8000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>308000</v>
+        <v>342047</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>-75.0%</t>
+          <t>-76.7%</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>-74.0%</t>
+          <t>-96.5%</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -555,38 +555,38 @@
         <v>100000</v>
       </c>
       <c r="D3" t="n">
-        <v>18785</v>
+        <v>19175</v>
       </c>
       <c r="E3" t="n">
-        <v>24874</v>
+        <v>24912</v>
       </c>
       <c r="F3" t="n">
-        <v>-6089</v>
+        <v>-5737</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>41395</v>
+        <v>41974</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>-54.6%</t>
+          <t>-54.3%</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>-142.9%</t>
+          <t>-139.0%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -607,38 +607,38 @@
         <v>800000</v>
       </c>
       <c r="D4" t="n">
-        <v>197067</v>
+        <v>220255</v>
       </c>
       <c r="E4" t="n">
-        <v>81119</v>
+        <v>91493</v>
       </c>
       <c r="F4" t="n">
-        <v>115947</v>
+        <v>128761</v>
       </c>
       <c r="G4" t="n">
         <v>10398</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>24.6%</t>
+          <t>27.5%</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>225139</v>
+        <v>237280</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>-12.5%</t>
+          <t>-7.2%</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>-33.4%</t>
+          <t>-30.3%</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -659,10 +659,10 @@
         <v>650000</v>
       </c>
       <c r="D5" t="n">
-        <v>23309</v>
+        <v>23347</v>
       </c>
       <c r="E5" t="n">
-        <v>69159</v>
+        <v>69197</v>
       </c>
       <c r="F5" t="n">
         <v>-45849</v>
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>284571</v>
+        <v>284590</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -711,38 +711,38 @@
         <v>700000</v>
       </c>
       <c r="D6" t="n">
-        <v>135037</v>
+        <v>143565</v>
       </c>
       <c r="E6" t="n">
-        <v>41016</v>
+        <v>41506</v>
       </c>
       <c r="F6" t="n">
-        <v>94020</v>
+        <v>102058</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>32521</v>
+        <v>34287</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>+315.2%</t>
+          <t>+318.7%</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>+414.9%</t>
+          <t>+411.0%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -763,38 +763,38 @@
         <v>550000</v>
       </c>
       <c r="D7" t="n">
-        <v>117462</v>
+        <v>132509</v>
       </c>
       <c r="E7" t="n">
-        <v>37267</v>
+        <v>37324</v>
       </c>
       <c r="F7" t="n">
-        <v>80195</v>
+        <v>95185</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>24.1%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>24.1%</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>182211</v>
+        <v>182703</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>-35.5%</t>
+          <t>-27.5%</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>-23.6%</t>
+          <t>-9.7%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -815,38 +815,38 @@
         <v>650000</v>
       </c>
       <c r="D8" t="n">
-        <v>169398</v>
+        <v>174229</v>
       </c>
       <c r="E8" t="n">
-        <v>15007</v>
+        <v>15136</v>
       </c>
       <c r="F8" t="n">
-        <v>154391</v>
+        <v>159093</v>
       </c>
       <c r="G8" t="n">
         <v>18796</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>26.1%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>114620</v>
+        <v>115582</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>+47.8%</t>
+          <t>+50.7%</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>+199.6%</t>
+          <t>+203.3%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -867,25 +867,25 @@
         <v>1700000</v>
       </c>
       <c r="D9" t="n">
-        <v>317341</v>
+        <v>366721</v>
       </c>
       <c r="E9" t="n">
         <v>53574</v>
       </c>
       <c r="F9" t="n">
-        <v>263767</v>
+        <v>313147</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -893,12 +893,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>+7.3%</t>
+          <t>+23.9%</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>+195.5%</t>
+          <t>+250.9%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -919,42 +919,42 @@
         <v>2000000</v>
       </c>
       <c r="D10" t="n">
-        <v>563265</v>
+        <v>603723</v>
       </c>
       <c r="E10" t="n">
         <v>19</v>
       </c>
       <c r="F10" t="n">
-        <v>563246</v>
+        <v>603704</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>41597</v>
+        <v>41995</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>+1254.1%</t>
+          <t>+1337.6%</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>+1528.0%</t>
+          <t>+1625.1%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>含普陀明细(517294元)</t>
+          <t>含普陀明细(557752元)</t>
         </is>
       </c>
     </row>
@@ -973,36 +973,36 @@
         <v>700000</v>
       </c>
       <c r="D11" t="n">
-        <v>214684</v>
+        <v>258878</v>
       </c>
       <c r="E11" t="n">
-        <v>8800</v>
+        <v>20800</v>
       </c>
       <c r="F11" t="n">
-        <v>205884</v>
+        <v>238078</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>187913</v>
+        <v>195509</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>+14.2%</t>
+          <t>+32.4%</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>+31.9%</t>
+          <t>+40.3%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1023,36 +1023,36 @@
         <v>450000</v>
       </c>
       <c r="D12" t="n">
-        <v>38614</v>
+        <v>52313</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>38605</v>
+        <v>52304</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>127784</v>
+        <v>137784</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>-69.8%</t>
+          <t>-62.0%</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>-59.8%</t>
+          <t>-50.6%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1073,36 +1073,36 @@
         <v>800000</v>
       </c>
       <c r="D13" t="n">
-        <v>223068</v>
+        <v>270755</v>
       </c>
       <c r="E13" t="n">
         <v>14056</v>
       </c>
       <c r="F13" t="n">
-        <v>209012</v>
+        <v>256699</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>33.8%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>33.8%</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>127816</v>
+        <v>177802</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>+74.5%</t>
+          <t>+52.3%</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>-700.9%</t>
+          <t>+3233.6%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1123,36 +1123,36 @@
         <v>850000</v>
       </c>
       <c r="D14" t="n">
-        <v>190041</v>
+        <v>216221</v>
       </c>
       <c r="E14" t="n">
-        <v>25781</v>
+        <v>30761</v>
       </c>
       <c r="F14" t="n">
-        <v>164260</v>
+        <v>185460</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>139236</v>
+        <v>150836</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>+36.5%</t>
+          <t>+43.3%</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>+72.0%</t>
+          <t>+73.2%</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1175,36 +1175,36 @@
         <v>450000</v>
       </c>
       <c r="D15" t="n">
-        <v>126918</v>
+        <v>134314</v>
       </c>
       <c r="E15" t="n">
         <v>299</v>
       </c>
       <c r="F15" t="n">
-        <v>126619</v>
+        <v>134015</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>29.8%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>29.8%</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>72983</v>
+        <v>100220</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>+73.9%</t>
+          <t>+34.0%</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>+120.7%</t>
+          <t>+58.4%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1225,23 +1225,23 @@
         <v>700000</v>
       </c>
       <c r="D16" t="n">
-        <v>166547</v>
+        <v>185595</v>
       </c>
       <c r="E16" t="n">
         <v>299</v>
       </c>
       <c r="F16" t="n">
-        <v>166248</v>
+        <v>185296</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>+28.1%</t>
+          <t>+42.8%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>+41.9%</t>
+          <t>+58.2%</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1277,36 +1277,36 @@
         <v>850000</v>
       </c>
       <c r="D17" t="n">
-        <v>123246</v>
+        <v>130765</v>
       </c>
       <c r="E17" t="n">
         <v>143178</v>
       </c>
       <c r="F17" t="n">
-        <v>-19931</v>
+        <v>-12412</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>142512</v>
+        <v>153510</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>-13.5%</t>
+          <t>-14.8%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>-118.7%</t>
+          <t>-110.6%</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1329,40 +1329,40 @@
         <v>800000</v>
       </c>
       <c r="D18" t="n">
-        <v>97456</v>
+        <v>110005</v>
       </c>
       <c r="E18" t="n">
         <v>16937</v>
       </c>
       <c r="F18" t="n">
-        <v>80519</v>
+        <v>93068</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>76217</v>
+        <v>90617</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>+27.9%</t>
+          <t>+21.4%</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>+895.2%</t>
+          <t>+313.8%</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>13642</v>
+        <v>15793</v>
       </c>
       <c r="N18" t="inlineStr"/>
     </row>
@@ -1401,16 +1401,16 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>15872</v>
+        <v>15891</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>+598.0%</t>
+          <t>+597.2%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>+503.9%</t>
+          <t>+503.2%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1431,23 +1431,23 @@
         <v>400000</v>
       </c>
       <c r="D20" t="n">
-        <v>50693</v>
+        <v>57489</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>10200</v>
       </c>
       <c r="F20" t="n">
-        <v>50693</v>
+        <v>47289</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="J20" t="n">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>+20.7%</t>
+          <t>+36.9%</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>+270.0%</t>
+          <t>+245.1%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -1477,38 +1477,38 @@
         <v>6150000</v>
       </c>
       <c r="D21" t="n">
-        <v>1055410</v>
+        <v>1159489</v>
       </c>
       <c r="E21" t="n">
-        <v>366021</v>
+        <v>407131</v>
       </c>
       <c r="F21" t="n">
-        <v>689387</v>
+        <v>752356</v>
       </c>
       <c r="G21" t="n">
         <v>76782</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1484340</v>
+        <v>1534346</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-28.9%</t>
+          <t>-24.4%</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-18.4%</t>
+          <t>-15.7%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -1525,44 +1525,44 @@
         <v>8260000</v>
       </c>
       <c r="D22" t="n">
-        <v>1905320</v>
+        <v>2130846</v>
       </c>
       <c r="E22" t="n">
-        <v>224655</v>
+        <v>251835</v>
       </c>
       <c r="F22" t="n">
-        <v>1680666</v>
+        <v>1879012</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1655887</v>
+        <v>1889501</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>+15.1%</t>
+          <t>+12.8%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>+38.0%</t>
+          <t>+29.6%</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>44852</v>
+        <v>47003</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>康博嘉5店(武汉4726,深圳13642,杭州23201,广州3283)</t>
+          <t>康博嘉5店(深圳15793,武汉4726,杭州23201,广州3283)</t>
         </is>
       </c>
     </row>
@@ -1577,44 +1577,44 @@
         <v>14410000</v>
       </c>
       <c r="D23" t="n">
-        <v>2960734</v>
+        <v>3290338</v>
       </c>
       <c r="E23" t="n">
-        <v>590677</v>
+        <v>658967</v>
       </c>
       <c r="F23" t="n">
-        <v>2370056</v>
+        <v>2631371</v>
       </c>
       <c r="G23" t="n">
         <v>76782</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>3140227</v>
+        <v>3423847</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>-5.7%</t>
+          <t>-3.9%</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>+14.9%</t>
+          <t>+12.3%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>含协同76782元 | 普陀明细517294元 | 康博嘉44852元 | 退费率20.0%</t>
+          <t>含协同76782元 | 普陀明细557752元 | 康博嘉47003元 | 退费率20.0%</t>
         </is>
       </c>
     </row>

</xml_diff>